<commit_message>
feat: 0,1 for backend and ML
</commit_message>
<xml_diff>
--- a/contacts.xlsx
+++ b/contacts.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:E2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -412,38 +412,30 @@
       <c r="D1" t="str">
         <v>Receiver Email</v>
       </c>
+      <c r="E1" t="str">
+        <v>Resume</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Ankita J.</v>
+        <v>Charul Sharma</v>
       </c>
       <c r="B2" t="str">
-        <v>Media.Net</v>
+        <v>Bloomscouts</v>
       </c>
       <c r="C2" t="str">
-        <v>SDE 1</v>
+        <v>Backend Developer</v>
       </c>
       <c r="D2" t="str">
-        <v>ankitajedi@gmail.com</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>Ankita J.</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Media.Net</v>
-      </c>
-      <c r="C3" t="str">
-        <v>SDE 1</v>
-      </c>
-      <c r="D3" t="str">
-        <v>ankita.j@media.net</v>
+        <v>𝗰𝗵𝗮𝗿𝘂𝗹@𝗯𝗹𝗼𝗼𝗺𝘀𝗰𝗼𝘂𝘁𝘀.𝗰𝗼𝗺</v>
+      </c>
+      <c r="E2" t="str">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: update mailer workflow and outreach contacts
</commit_message>
<xml_diff>
--- a/contacts.xlsx
+++ b/contacts.xlsx
@@ -1,52 +1,29 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
+  <definedNames/>
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-  </numFmts>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
   <fonts count="1">
     <font>
-      <sz val="12"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="12"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -65,13 +42,80 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -396,46 +440,214 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="str">
-        <v>Receiver Name</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Company Name</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Job Link</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Receiver Email</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Resume</v>
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Receiver Name</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Company Name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Job Link</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Receiver Email</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Resume</t>
+        </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="str">
-        <v>Charul Sharma</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Bloomscouts</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Backend Developer</v>
-      </c>
-      <c r="D2" t="str">
-        <v>𝗰𝗵𝗮𝗿𝘂𝗹@𝗯𝗹𝗼𝗼𝗺𝘀𝗰𝗼𝘂𝘁𝘀.𝗰𝗼𝗺</v>
-      </c>
-      <c r="E2" t="str">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Saranga </t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Myntra</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Senior Software Engineer</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>saranga.deshmukh@myntra.com</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Gourav Rusiya</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>gouravrusiya.lnct@gmail.com</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
         <v>0</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Nehlata Pandey</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Recro</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Applied ML Scientist – Voice AI (Bengaluru | WFO)</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>nehlata.pandey@recro.io</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Madhu Kiran</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Myntra</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>ML Engineer</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>madhu.kiran@myntra.com</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Vara Lakshmi Addepalli</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Tekion</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Software Engineer II-Backend</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>vara96addepalli@gmail.com</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Dheeraj Gupta</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>American Express</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Software Engineer 2</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>dheerajgupta2897@gmail.com</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Hiring Team</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Zypp Electric</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>SDE-2 (Backend - Java) | 3-5 yrs | Gurugram WFO</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>hirings@zypp.app</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E2"/>
-  </ignoredErrors>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>